<commit_message>
updated side_effect_counts from code chunk #12
top 30 side effects with DBID counts and DT counts
</commit_message>
<xml_diff>
--- a/side_effect_count.xlsx
+++ b/side_effect_count.xlsx
@@ -465,7 +465,9 @@
       <c r="D2" t="n">
         <v>795</v>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>736</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -480,9 +482,11 @@
         <v>2601</v>
       </c>
       <c r="D3" t="n">
-        <v>906</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
+        <v>908</v>
+      </c>
+      <c r="E3" t="n">
+        <v>834</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -497,9 +501,11 @@
         <v>2416</v>
       </c>
       <c r="D4" t="n">
-        <v>852</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
+        <v>853</v>
+      </c>
+      <c r="E4" t="n">
+        <v>788</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -514,9 +520,11 @@
         <v>2403</v>
       </c>
       <c r="D5" t="n">
-        <v>815</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>816</v>
+      </c>
+      <c r="E5" t="n">
+        <v>753</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -531,9 +539,11 @@
         <v>2345</v>
       </c>
       <c r="D6" t="n">
-        <v>824</v>
-      </c>
-      <c r="E6" t="inlineStr"/>
+        <v>825</v>
+      </c>
+      <c r="E6" t="n">
+        <v>758</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -550,7 +560,9 @@
       <c r="D7" t="n">
         <v>709</v>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>667</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -565,9 +577,11 @@
         <v>2200</v>
       </c>
       <c r="D8" t="n">
-        <v>746</v>
-      </c>
-      <c r="E8" t="inlineStr"/>
+        <v>747</v>
+      </c>
+      <c r="E8" t="n">
+        <v>690</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -582,9 +596,11 @@
         <v>2049</v>
       </c>
       <c r="D9" t="n">
-        <v>727</v>
-      </c>
-      <c r="E9" t="inlineStr"/>
+        <v>726</v>
+      </c>
+      <c r="E9" t="n">
+        <v>669</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -601,7 +617,9 @@
       <c r="D10" t="n">
         <v>678</v>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>623</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -618,7 +636,9 @@
       <c r="D11" t="n">
         <v>637</v>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>586</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -633,9 +653,11 @@
         <v>1744</v>
       </c>
       <c r="D12" t="n">
-        <v>615</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
+        <v>616</v>
+      </c>
+      <c r="E12" t="n">
+        <v>570</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -652,7 +674,9 @@
       <c r="D13" t="n">
         <v>603</v>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>559</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -667,9 +691,11 @@
         <v>1676</v>
       </c>
       <c r="D14" t="n">
-        <v>824</v>
-      </c>
-      <c r="E14" t="inlineStr"/>
+        <v>825</v>
+      </c>
+      <c r="E14" t="n">
+        <v>762</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -686,7 +712,9 @@
       <c r="D15" t="n">
         <v>561</v>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>515</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -701,9 +729,11 @@
         <v>1624</v>
       </c>
       <c r="D16" t="n">
-        <v>582</v>
-      </c>
-      <c r="E16" t="inlineStr"/>
+        <v>581</v>
+      </c>
+      <c r="E16" t="n">
+        <v>547</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -718,9 +748,11 @@
         <v>1560</v>
       </c>
       <c r="D17" t="n">
-        <v>578</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
+        <v>576</v>
+      </c>
+      <c r="E17" t="n">
+        <v>546</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -735,9 +767,11 @@
         <v>1536</v>
       </c>
       <c r="D18" t="n">
-        <v>555</v>
-      </c>
-      <c r="E18" t="inlineStr"/>
+        <v>554</v>
+      </c>
+      <c r="E18" t="n">
+        <v>521</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -754,7 +788,9 @@
       <c r="D19" t="n">
         <v>567</v>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>537</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -771,7 +807,9 @@
       <c r="D20" t="n">
         <v>543</v>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>506</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -788,7 +826,9 @@
       <c r="D21" t="n">
         <v>517</v>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>480</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -805,7 +845,9 @@
       <c r="D22" t="n">
         <v>545</v>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>515</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -820,9 +862,11 @@
         <v>1434</v>
       </c>
       <c r="D23" t="n">
-        <v>469</v>
-      </c>
-      <c r="E23" t="inlineStr"/>
+        <v>468</v>
+      </c>
+      <c r="E23" t="n">
+        <v>423</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -837,9 +881,11 @@
         <v>1426</v>
       </c>
       <c r="D24" t="n">
-        <v>522</v>
-      </c>
-      <c r="E24" t="inlineStr"/>
+        <v>523</v>
+      </c>
+      <c r="E24" t="n">
+        <v>489</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -854,9 +900,11 @@
         <v>1388</v>
       </c>
       <c r="D25" t="n">
-        <v>548</v>
-      </c>
-      <c r="E25" t="inlineStr"/>
+        <v>547</v>
+      </c>
+      <c r="E25" t="n">
+        <v>514</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -871,9 +919,11 @@
         <v>1326</v>
       </c>
       <c r="D26" t="n">
-        <v>498</v>
-      </c>
-      <c r="E26" t="inlineStr"/>
+        <v>497</v>
+      </c>
+      <c r="E26" t="n">
+        <v>468</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -888,9 +938,11 @@
         <v>1298</v>
       </c>
       <c r="D27" t="n">
-        <v>492</v>
-      </c>
-      <c r="E27" t="inlineStr"/>
+        <v>491</v>
+      </c>
+      <c r="E27" t="n">
+        <v>462</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -907,7 +959,9 @@
       <c r="D28" t="n">
         <v>468</v>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>440</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -922,9 +976,11 @@
         <v>1268</v>
       </c>
       <c r="D29" t="n">
-        <v>461</v>
-      </c>
-      <c r="E29" t="inlineStr"/>
+        <v>460</v>
+      </c>
+      <c r="E29" t="n">
+        <v>430</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -941,7 +997,9 @@
       <c r="D30" t="n">
         <v>462</v>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>441</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -958,7 +1016,9 @@
       <c r="D31" t="n">
         <v>543</v>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>507</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>